<commit_message>
continuing to encounter latex rendering errors, will try to switch to using openstax api
</commit_message>
<xml_diff>
--- a/trig_examples.xlsx
+++ b/trig_examples.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -553,7 +553,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Using the formula for the cosine of the difference of two angles, find the exact value of cos⁡(5⁢𝜋4−𝜋6).cos⁡(5⁢π4−π6).cos(5π4−π6).</t>
+          <t>Using the formula for the cosine of the difference of two angles, find the exact value of cos⁡(5⁢π4−π6).cos(5π4−π6).</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -581,11 +581,7 @@
           <t>problem</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Finding the Exact Value Using the Formula for the Sum of Two Angles for Cosine</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -613,7 +609,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Find the exact value of cos⁡(75∘).cos⁡(75∘).cos(75∘).</t>
+          <t>Find the exact value of cos⁡(π3−π4).cos(π3−π4).</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -643,14 +639,10 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Using Sum and Difference Identities to Evaluate the Difference of Angles</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Use the sum and difference identities to evaluate the difference of the angles and show that part a equals part b.</t>
-        </is>
-      </c>
+          <t>Finding the Exact Value Using the Formula for the Sum of Two Angles for Cosine</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
@@ -675,7 +667,11 @@
           <t>step</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Find the exact value of cos⁡(75∘).cos(75∘).</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
@@ -693,12 +689,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>trig3</t>
+          <t>trig4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>step</t>
+          <t>problem</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -724,12 +720,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>problem</t>
+          <t>step</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Finding the Exact Value of an Expression Involving an Inverse Trigonometric Function</t>
+          <t>Find the exact value of cos⁡(105∘).cos(105∘).</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -749,20 +745,24 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>trig4</t>
+          <t>trig5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>step</t>
+          <t>problem</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Find the exact value of sin⁡(cos−112+sin−135).sin⁡(cos−112+sin−135).sin(cos−112+sin−135).</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
+          <t>Using Sum and Difference Identities to Evaluate the Difference of Angles</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Use the sum and difference identities to evaluate the difference of the angles and show that part a equals part b.</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -784,12 +784,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>problem</t>
+          <t>step</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Finding the Exact Value of an Expression Involving Tangent</t>
+          <t>sin⁡(45∘−30∘)sin(45∘−30∘)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -819,7 +819,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Find the exact value of tan⁡(𝜋6+𝜋4).tan⁡(π6+π4).tan(π6+π4).</t>
+          <t>sin⁡(135∘−120∘)sin(135∘−120∘)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -849,14 +849,10 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Finding Multiple Sums and Differences of Angles</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Given sin⁡𝛼=35,0&lt;𝛼&lt;𝜋2,cos⁡𝛽=−513,𝜋&lt;𝛽&lt;3⁢𝜋2,sin⁡α=35,0&lt;α&lt;π2,cos⁡β=−513,π&lt;β&lt;3⁢π2,sinα=35,0&lt;α&lt;π2,cosβ=−513,π&lt;β&lt;3π2, find</t>
-        </is>
-      </c>
+          <t>Finding the Exact Value of an Expression Involving an Inverse Trigonometric Function</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
@@ -881,7 +877,11 @@
           <t>step</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Find the exact value of sin⁡(cos−112+sin−135).sin(cos−112+sin−135).</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -899,15 +899,19 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>trig6</t>
+          <t>trig7</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>step</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Finding the Exact Value of an Expression Involving Tangent</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
@@ -925,7 +929,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>trig6</t>
+          <t>trig7</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -933,7 +937,11 @@
           <t>step</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Find the exact value of tan⁡(π6+π4).tan(π6+π4).</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
@@ -951,12 +959,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>trig6</t>
+          <t>trig8</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>step</t>
+          <t>problem</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -977,17 +985,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>trig7</t>
+          <t>trig8</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>problem</t>
+          <t>step</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Finding a Cofunction with the Same Value as the Given Expression</t>
+          <t>Find the exact value of tan⁡(2⁢π3+π4).tan(2π3+π4).</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1007,20 +1015,24 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>trig7</t>
+          <t>trig9</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>step</t>
+          <t>problem</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Write tan𝜋9tanπ9tanπ9 in terms of its cofunction.</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
+          <t>Finding Multiple Sums and Differences of Angles</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Given sin⁡α=35,0&lt;α&lt;π2,cos⁡β=−513,π&lt;β&lt;3⁢π2,sinα=35,0&lt;α&lt;π2,cosβ=−513,π&lt;β&lt;3π2, find</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
@@ -1037,17 +1049,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>trig8</t>
+          <t>trig9</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>problem</t>
+          <t>step</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Verifying an Identity Involving Sine</t>
+          <t>sin⁡(α+β)sin(α+β)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1067,7 +1079,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>trig8</t>
+          <t>trig9</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1077,7 +1089,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Verify the identity sin⁡(𝛼+𝛽)+sin⁡(𝛼−𝛽)=2sin⁡𝛼⁢cos⁡𝛽.sin⁡(α+β)+sin⁡(α−β)=2sin⁡α⁢cos⁡β.sin(α+β)+sin(α−β)=2sinαcosβ.</t>
+          <t>cos⁡(α+β)cos(α+β)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1102,12 +1114,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>problem</t>
+          <t>step</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Verifying an Identity Involving Tangent</t>
+          <t>tan⁡(α+β)tan(α+β)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1137,7 +1149,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Verify the following identity.</t>
+          <t>tan⁡(α−β)tan(α−β)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1167,7 +1179,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Using Sum and Difference Formulas to Solve an Application Problem</t>
+          <t>Finding a Cofunction with the Same Value as the Given Expression</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1197,7 +1209,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Let 𝐿1L1L1 and 𝐿2L2L2 denote two non-vertical intersecting lines, and let 𝜃θθ denote the acute angle between 𝐿1L1L1 and 𝐿2.L2.L2. See Figure 7. Show that where 𝑚1m1m1 and 𝑚2m2m2 are the slopes of 𝐿1L1L1 and 𝐿2L2L2 respectively. (Hint: Use the fact that tan⁡𝜃1=𝑚1tan⁡θ1=m1tanθ1=m1 and tan⁡𝜃2=𝑚2.tan⁡θ2=m2.tanθ2=m2. ) Figure 7</t>
+          <t>Write tanπ9tanπ9 in terms of its cofunction.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1225,11 +1237,7 @@
           <t>problem</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Investigating a Guy-wire Problem</t>
-        </is>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -1257,7 +1265,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>For a climbing wall, a guy-wire 𝑅RR is attached 47 feet high on a vertical pole. Added support is provided by another guy-wire 𝑆SS attached 40 feet above ground on the same pole. If the wires are attached to the ground 50 feet from the pole, find the angle 𝛼αα between the wires. See Figure 8. Figure 8</t>
+          <t>Write sinπ7sinπ7 in terms of its cofunction.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1274,6 +1282,3438 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>trig12</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Verifying an Identity Involving Sine</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>trig12</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Verify the identity sin⁡(α+β)+sin⁡(α−β)=2sin⁡α⁢cos⁡β.sin(α+β)+sin(α−β)=2sinαcosβ.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>trig13</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Verifying an Identity Involving Tangent</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>trig13</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Verify the following identity. sin⁡(α−β)cos⁡α⁢cos⁡β=tan⁡α−tan⁡βsin(α−β)cosαcosβ=tanα−tanβ</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>trig14</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>trig14</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Verify the identity: tan⁡(π−θ)=−tan⁡θ.tan(π−θ)=−tanθ.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>trig15</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Using Sum and Difference Formulas to Solve an Application Problem</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>trig15</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Let L1L1 and L2L2 denote two non-vertical intersecting lines, and let θθ denote the acute angle between L1L1 and L2.L2. See Figure 7. Show that tan⁡θ=m2−m11+m1⁢m2tanθ=m2−m11+m1m2 where m1m1 and m2m2 are the slopes of L1L1 and L2L2 respectively. (Hint: Use the fact that tan⁡θ1=m1tanθ1=m1 and tan⁡θ2=m2.tanθ2=m2. ) Figure 7</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>trig16</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Investigating a Guy-wire Problem</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>trig16</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>For a climbing wall, a guy-wire RR is attached 47 feet high on a vertical pole. Added support is provided by another guy-wire SS attached 40 feet above ground on the same pole. If the wires are attached to the ground 50 feet from the pole, find the angle αα between the wires. See Figure 8. Figure 8</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>trig17</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>trig17</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1. Explain the basis for the cofunction identities and when they apply.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>trig18</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>trig18</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2. Is there only one way to evaluate cos⁡(5⁢π4)?cos(5π4)? Explain how to set up the solution in two different ways, and then compute to make sure they give the same answer.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>trig19</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>trig19</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>3. Explain to someone who has forgotten the even-odd properties of sinusoidal functions how the addition and subtraction formulas can determine this characteristic for f⁡(x)=sin⁡(x)f(x)=sin(x) and g⁡(x)=cos⁡(x).g(x)=cos(x). (Hint: 0−x=−x0−x=−x )</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>trig20</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>trig20</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>4. cos⁡(7⁢π12)cos(7π12)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>trig21</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>trig21</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>5. cos⁡(π12)cos(π12)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>trig22</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>trig22</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>6. sin⁡(5⁢π12)sin(5π12)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>trig23</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>trig23</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>7. sin⁡(11⁢π12)sin(11π12)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>trig24</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>trig24</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>8. tan⁡(−π12)tan(−π12)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>trig25</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>trig25</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>9. tan⁡(19⁢π12)tan(19π12)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>trig26</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>trig26</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>10. sin⁡(x+11⁢π6)sin(x+11π6)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>trig27</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>trig27</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>11. sin⁡(x−3⁢π4)sin(x−3π4)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>trig28</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>trig28</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>12. cos⁡(x−5⁢π6)cos(x−5π6)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>trig29</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>trig29</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>13. cos⁡(x+2⁢π3)cos(x+2π3)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>trig30</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>trig30</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>14. csc⁡(π2−t)csc(π2−t)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>trig31</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>trig31</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>15. sec⁡(π2−θ)sec(π2−θ)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>trig32</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>trig32</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>16. cot⁡(π2−x)cot(π2−x)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>trig33</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>trig33</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>17. tan⁡(π2−x)tan(π2−x)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
+      <c r="P71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>trig34</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>trig34</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>18. sin⁡(2⁢x)⁢cos⁡(5⁢x)−sin⁡(5⁢x)⁢cos⁡(2⁢x)sin(2x)cos(5x)−sin(5x)cos(2x)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>trig35</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>trig35</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>19. tan⁡(32⁢x)−tan⁡(75⁢x)1+tan⁡(32⁢x)⁢tan⁡(75⁢x)tan(32x)−tan(75x)1+tan(32x)tan(75x)</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
+      <c r="P75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>trig36</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
+      <c r="P76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>trig36</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>20. Given that sin⁡a=23sina=23 and cos⁡b=−14,cosb=−14, with aa and bb both in the interval [π2,π),[π2,π), find sin⁡(a+b)sin(a+b) and cos⁡(a−b).cos(a−b).</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
+      <c r="P77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>trig37</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
+      <c r="P78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>trig37</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>21. Given that sin⁡a=45,sina=45, and cos⁡b=13,cosb=13, with aa and bb both in the interval [0,π2),[0,π2), find sin⁡(a−b)sin(a−b) and cos⁡(a+b).cos(a+b).</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr"/>
+      <c r="P79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>trig38</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
+      <c r="P80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>trig38</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>22. sin⁡(cos−1⁡(0)−cos−1⁡(12))sin(cos−1(0)−cos−1(12))</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr"/>
+      <c r="P81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>trig39</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr"/>
+      <c r="P82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>trig39</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>23. cos⁡(cos−1⁡(22)+sin−1⁡(32))cos(cos−1(22)+sin−1(32))</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr"/>
+      <c r="P83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>trig40</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
+      <c r="P84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>trig40</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>24. tan⁡(sin−1⁡(12)−cos−1⁡(12))tan(sin−1(12)−cos−1(12))</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr"/>
+      <c r="P85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>trig41</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
+      <c r="P86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>trig41</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>25. cos⁡(π2−x)cos(π2−x)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
+      <c r="P87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>trig42</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
+      <c r="P88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>trig42</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>26. sin⁡(π−x)sin(π−x)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr"/>
+      <c r="P89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>trig43</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr"/>
+      <c r="P90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>trig43</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>27. tan⁡(π3+x)tan(π3+x)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr"/>
+      <c r="P91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>trig44</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr"/>
+      <c r="P92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>trig44</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>28. sin⁡(π3+x)sin(π3+x)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr"/>
+      <c r="P93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>trig45</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr"/>
+      <c r="P94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>trig45</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>29. tan⁡(π4−x)tan(π4−x)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr"/>
+      <c r="P95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>trig46</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr"/>
+      <c r="P96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>trig46</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>30. cos⁡(7⁢π6+x)cos(7π6+x)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr"/>
+      <c r="P97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>trig47</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr"/>
+      <c r="P98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>trig47</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>31. sin⁡(π4+x)sin(π4+x)</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr"/>
+      <c r="P99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>trig48</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="inlineStr"/>
+      <c r="O100" t="inlineStr"/>
+      <c r="P100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>trig48</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>32. cos⁡(5⁢π4+x)cos(5π4+x)</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
+      <c r="N101" t="inlineStr"/>
+      <c r="O101" t="inlineStr"/>
+      <c r="P101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>trig49</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
+      <c r="N102" t="inlineStr"/>
+      <c r="O102" t="inlineStr"/>
+      <c r="P102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>trig49</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>33. f⁡(x)=sin⁡(4⁢x)−sin⁡(3⁢x)⁢cos⁡xf(x)=sin(4x)−sin(3x)cosx , g⁡(x)=sin⁡x⁢cos⁡(3⁢x)g(x)=sinxcos(3x)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
+      <c r="N103" t="inlineStr"/>
+      <c r="O103" t="inlineStr"/>
+      <c r="P103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>trig50</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr"/>
+      <c r="N104" t="inlineStr"/>
+      <c r="O104" t="inlineStr"/>
+      <c r="P104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>trig50</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>34. f⁡(x)=cos⁡(4⁢x)+sin⁡x⁢sin⁡(3⁢x),g⁡(x)=−cos⁡x⁢cos⁡(3⁢x)f(x)=cos(4x)+sinxsin(3x),g(x)=−cosxcos(3x)</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr"/>
+      <c r="N105" t="inlineStr"/>
+      <c r="O105" t="inlineStr"/>
+      <c r="P105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>trig51</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="inlineStr"/>
+      <c r="N106" t="inlineStr"/>
+      <c r="O106" t="inlineStr"/>
+      <c r="P106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>trig51</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>35. f⁡(x)=sin⁡(3⁢x)⁢cos⁡(6⁢x)f(x)=sin(3x)cos(6x) , g⁡(x)=−sin⁡(3⁢x)⁢cos⁡(6⁢x)g(x)=−sin(3x)cos(6x)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr"/>
+      <c r="N107" t="inlineStr"/>
+      <c r="O107" t="inlineStr"/>
+      <c r="P107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>trig52</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="inlineStr"/>
+      <c r="N108" t="inlineStr"/>
+      <c r="O108" t="inlineStr"/>
+      <c r="P108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>trig52</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>36. f⁡(x)=sin⁡(4⁢x)f(x)=sin(4x) , g⁡(x)=sin⁡(5⁢x)⁢cos⁡x−cos⁡(5⁢x)⁢sin⁡xg(x)=sin(5x)cosx−cos(5x)sinx</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr"/>
+      <c r="N109" t="inlineStr"/>
+      <c r="O109" t="inlineStr"/>
+      <c r="P109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>trig53</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr"/>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="inlineStr"/>
+      <c r="N110" t="inlineStr"/>
+      <c r="O110" t="inlineStr"/>
+      <c r="P110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>trig53</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>37. f⁡(x)=sin⁡(2⁢x)f(x)=sin(2x) , g⁡(x)=2sin⁡x⁢cos⁡xg(x)=2sinxcosx</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr"/>
+      <c r="N111" t="inlineStr"/>
+      <c r="O111" t="inlineStr"/>
+      <c r="P111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>trig54</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr"/>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr"/>
+      <c r="N112" t="inlineStr"/>
+      <c r="O112" t="inlineStr"/>
+      <c r="P112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>trig54</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>38. f⁡(θ)=cos⁡(2⁢θ)f(θ)=cos(2θ) , g⁡(θ)=cos2⁡θ−sin2⁡θg(θ)=cos2θ−sin2θ</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr"/>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr"/>
+      <c r="P113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>trig55</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr"/>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr"/>
+      <c r="M114" t="inlineStr"/>
+      <c r="N114" t="inlineStr"/>
+      <c r="O114" t="inlineStr"/>
+      <c r="P114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>trig55</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>39. f⁡(θ)=tan⁡(2⁢θ)f(θ)=tan(2θ) , g⁡(θ)=tan⁡θ1+tan2⁡θg(θ)=tanθ1+tan2θ</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr"/>
+      <c r="N115" t="inlineStr"/>
+      <c r="O115" t="inlineStr"/>
+      <c r="P115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>trig56</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr"/>
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr"/>
+      <c r="N116" t="inlineStr"/>
+      <c r="O116" t="inlineStr"/>
+      <c r="P116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>trig56</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>40. f⁡(x)=sin⁡(3⁢x)⁢sin⁡xf(x)=sin(3x)sinx , g⁡(x)=sin2⁡(2⁢x)⁢cos2⁡x−cos2⁡(2⁢x)⁢sin2⁡xg(x)=sin2(2x)cos2x−cos2(2x)sin2x</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr"/>
+      <c r="N117" t="inlineStr"/>
+      <c r="O117" t="inlineStr"/>
+      <c r="P117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>trig57</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr"/>
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
+      <c r="N118" t="inlineStr"/>
+      <c r="O118" t="inlineStr"/>
+      <c r="P118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>trig57</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>41. f⁡(x)=tan⁡(−x)f(x)=tan(−x) , g⁡(x)=tan⁡x−tan⁡(2⁢x)1−tan⁡x⁢tan⁡(2⁢x)g(x)=tanx−tan(2x)1−tanxtan(2x)</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr"/>
+      <c r="N119" t="inlineStr"/>
+      <c r="O119" t="inlineStr"/>
+      <c r="P119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>trig58</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr"/>
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr"/>
+      <c r="N120" t="inlineStr"/>
+      <c r="O120" t="inlineStr"/>
+      <c r="P120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>trig58</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>42. sin⁡(75∘)sin(75∘)</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="inlineStr"/>
+      <c r="O121" t="inlineStr"/>
+      <c r="P121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>trig59</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr"/>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr"/>
+      <c r="N122" t="inlineStr"/>
+      <c r="O122" t="inlineStr"/>
+      <c r="P122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>trig59</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>43. sin⁡(195∘)sin(195∘)</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="inlineStr"/>
+      <c r="N123" t="inlineStr"/>
+      <c r="O123" t="inlineStr"/>
+      <c r="P123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>trig60</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr"/>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="inlineStr"/>
+      <c r="N124" t="inlineStr"/>
+      <c r="O124" t="inlineStr"/>
+      <c r="P124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>trig60</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>44. cos⁡(165∘)cos(165∘)</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr"/>
+      <c r="N125" t="inlineStr"/>
+      <c r="O125" t="inlineStr"/>
+      <c r="P125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>trig61</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr"/>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="inlineStr"/>
+      <c r="N126" t="inlineStr"/>
+      <c r="O126" t="inlineStr"/>
+      <c r="P126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>trig61</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>45. cos⁡(345∘)cos(345∘)</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="inlineStr"/>
+      <c r="N127" t="inlineStr"/>
+      <c r="O127" t="inlineStr"/>
+      <c r="P127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>trig62</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr"/>
+      <c r="D128" t="inlineStr"/>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr"/>
+      <c r="L128" t="inlineStr"/>
+      <c r="M128" t="inlineStr"/>
+      <c r="N128" t="inlineStr"/>
+      <c r="O128" t="inlineStr"/>
+      <c r="P128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>trig62</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>46. tan⁡(−15∘)tan(−15∘)</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
+      <c r="M129" t="inlineStr"/>
+      <c r="N129" t="inlineStr"/>
+      <c r="O129" t="inlineStr"/>
+      <c r="P129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>trig63</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr"/>
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr"/>
+      <c r="L130" t="inlineStr"/>
+      <c r="M130" t="inlineStr"/>
+      <c r="N130" t="inlineStr"/>
+      <c r="O130" t="inlineStr"/>
+      <c r="P130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>trig63</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>47. tan⁡(x+π4)=tan⁡x+11−tan⁡xtan(x+π4)=tanx+11−tanx</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr"/>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
+      <c r="L131" t="inlineStr"/>
+      <c r="M131" t="inlineStr"/>
+      <c r="N131" t="inlineStr"/>
+      <c r="O131" t="inlineStr"/>
+      <c r="P131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>trig64</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr"/>
+      <c r="D132" t="inlineStr"/>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr"/>
+      <c r="L132" t="inlineStr"/>
+      <c r="M132" t="inlineStr"/>
+      <c r="N132" t="inlineStr"/>
+      <c r="O132" t="inlineStr"/>
+      <c r="P132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>trig64</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>48. tan⁡(a+b)tan⁡(a−b)=sin⁡a⁢cos⁡a+sin⁡b⁢cos⁡bsin⁡a⁢cos⁡a−sin⁡b⁢cos⁡btan(a+b)tan(a−b)=sinacosa+sinbcosbsinacosa−sinbcosb</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr"/>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr"/>
+      <c r="L133" t="inlineStr"/>
+      <c r="M133" t="inlineStr"/>
+      <c r="N133" t="inlineStr"/>
+      <c r="O133" t="inlineStr"/>
+      <c r="P133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>trig65</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr"/>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr"/>
+      <c r="L134" t="inlineStr"/>
+      <c r="M134" t="inlineStr"/>
+      <c r="N134" t="inlineStr"/>
+      <c r="O134" t="inlineStr"/>
+      <c r="P134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>trig65</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>49. cos⁡(a+b)cos⁡a⁢cos⁡b=1−tan⁡a⁢tan⁡bcos(a+b)cosacosb=1−tanatanb</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr"/>
+      <c r="L135" t="inlineStr"/>
+      <c r="M135" t="inlineStr"/>
+      <c r="N135" t="inlineStr"/>
+      <c r="O135" t="inlineStr"/>
+      <c r="P135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>trig66</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr"/>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr"/>
+      <c r="L136" t="inlineStr"/>
+      <c r="M136" t="inlineStr"/>
+      <c r="N136" t="inlineStr"/>
+      <c r="O136" t="inlineStr"/>
+      <c r="P136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>trig66</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>50. cos⁡(x+y)⁢cos⁡(x−y)=cos2⁡x−sin2⁡ycos(x+y)cos(x−y)=cos2x−sin2y</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr"/>
+      <c r="L137" t="inlineStr"/>
+      <c r="M137" t="inlineStr"/>
+      <c r="N137" t="inlineStr"/>
+      <c r="O137" t="inlineStr"/>
+      <c r="P137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>trig67</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr"/>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr"/>
+      <c r="L138" t="inlineStr"/>
+      <c r="M138" t="inlineStr"/>
+      <c r="N138" t="inlineStr"/>
+      <c r="O138" t="inlineStr"/>
+      <c r="P138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>trig67</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>51. cos⁡(x+h)−cos⁡xh=cos⁡x⁢cos⁡h−1h−sin⁡x⁢sin⁡hhcos(x+h)−cosxh=cosxcosh−1h−sinxsinhh</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
+      <c r="L139" t="inlineStr"/>
+      <c r="M139" t="inlineStr"/>
+      <c r="N139" t="inlineStr"/>
+      <c r="O139" t="inlineStr"/>
+      <c r="P139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>trig68</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr"/>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
+      <c r="L140" t="inlineStr"/>
+      <c r="M140" t="inlineStr"/>
+      <c r="N140" t="inlineStr"/>
+      <c r="O140" t="inlineStr"/>
+      <c r="P140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>trig68</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>52. tan⁡(u+v)=tan⁡u+tan⁡v1−tan⁡u⁢tan⁡vtan(u+v)=tanu+tanv1−tanutanv</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr"/>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="inlineStr"/>
+      <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr"/>
+      <c r="P141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>trig69</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr"/>
+      <c r="D142" t="inlineStr"/>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr"/>
+      <c r="L142" t="inlineStr"/>
+      <c r="M142" t="inlineStr"/>
+      <c r="N142" t="inlineStr"/>
+      <c r="O142" t="inlineStr"/>
+      <c r="P142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>trig69</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>53. tan⁡(u−v)=tan⁡u−tan⁡v1+tan⁡u⁢tan⁡vtan(u−v)=tanu−tanv1+tanutanv</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr"/>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr"/>
+      <c r="L143" t="inlineStr"/>
+      <c r="M143" t="inlineStr"/>
+      <c r="N143" t="inlineStr"/>
+      <c r="O143" t="inlineStr"/>
+      <c r="P143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>trig70</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr"/>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr"/>
+      <c r="L144" t="inlineStr"/>
+      <c r="M144" t="inlineStr"/>
+      <c r="N144" t="inlineStr"/>
+      <c r="O144" t="inlineStr"/>
+      <c r="P144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>trig70</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>54. tan⁡(x+y)1+tan⁡x⁢tan⁡x=tan⁡x+tan⁡y1−tan2⁡x⁢tan2⁡ytan(x+y)1+tanxtanx=tanx+tany1−tan2xtan2y</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr"/>
+      <c r="L145" t="inlineStr"/>
+      <c r="M145" t="inlineStr"/>
+      <c r="N145" t="inlineStr"/>
+      <c r="O145" t="inlineStr"/>
+      <c r="P145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>trig71</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr"/>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr"/>
+      <c r="L146" t="inlineStr"/>
+      <c r="M146" t="inlineStr"/>
+      <c r="N146" t="inlineStr"/>
+      <c r="O146" t="inlineStr"/>
+      <c r="P146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>trig71</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>55. If α,β,α, β, and γγ are angles in the same triangle, then prove or disprove sin⁡(α+β)=sin⁡γ.sin(α+β)=sinγ.</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr"/>
+      <c r="M147" t="inlineStr"/>
+      <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr"/>
+      <c r="P147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>trig72</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>problem</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr"/>
+      <c r="L148" t="inlineStr"/>
+      <c r="M148" t="inlineStr"/>
+      <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr"/>
+      <c r="P148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>trig72</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>56. If α,β,α,β, and γγ are angles in the same triangle, then prove or disprove tan⁡α+tan⁡β+tan⁡γ=tan⁡α⁢tan⁡β⁢tan⁡γtanα+tanβ+tanγ=tanαtanβtanγ</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr"/>
+      <c r="L149" t="inlineStr"/>
+      <c r="M149" t="inlineStr"/>
+      <c r="N149" t="inlineStr"/>
+      <c r="O149" t="inlineStr"/>
+      <c r="P149" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added prompting for gemini 2.0 flash
</commit_message>
<xml_diff>
--- a/trig_examples.xlsx
+++ b/trig_examples.xlsx
@@ -553,7 +553,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Using the formula for the cosine of the difference of two angles, find the exact value of $cos(\frac{5\pi }{4}-\frac{\pi }{6}).cos(\frac{5\pi }{4}-\frac{\pi }{6}).$</t>
+          <t>Using the formula for the cosine of the difference of two angles, find the exact value of $$cos(\frac{5π}{4}−\frac{π}{6}).$$</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -613,7 +613,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Find the exact value of $cos(75^{∘}).cos(75^{∘}).$</t>
+          <t>Find the exact value of $$cos(75^{∘}).$$</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -677,7 +677,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>$sin(45^{∘}-30^{∘})sin(45^{∘}-30^{∘})$</t>
+          <t>$$sin(45^{∘}−30^{∘})$$</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -707,7 +707,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>$sin(135^{∘}-120^{∘})sin(135^{∘}-120^{∘})$</t>
+          <t>$$sin(135^{∘}−120^{∘})$$</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -767,7 +767,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Find the exact value of $sin(cos^{-1}\frac{1}{2}+sin^{-1}\frac{3}{5}).sin(cos^{-1}\frac{1}{2}+sin^{-1}\frac{3}{5}).$</t>
+          <t>Find the exact value of $$sin(cos^{−1}\frac{1}{2}+sin^{−1}\frac{3}{5}).$$</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -827,7 +827,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Find the exact value of $tan(\frac{\pi }{6}+\frac{\pi }{4}).tan(\frac{\pi }{6}+\frac{\pi }{4}).$</t>
+          <t>Find the exact value of $$tan(\frac{π}{6}+\frac{π}{4}).$$</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -862,7 +862,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Given $sinα=\frac{3}{5},0&lt;α&lt;\frac{\pi }{2},cosβ=-\frac{5}{13},\pi &lt;β&lt;\frac{3\pi }{2},sinα=\frac{3}{5},0&lt;α&lt;\frac{\pi }{2},cosβ=-\frac{5}{13},\pi &lt;β&lt;\frac{3\pi }{2},$ find</t>
+          <t>Given $$sinα=\frac{3}{5},0&lt;α&lt;\frac{π}{2},cosβ=−\frac{5}{13},π&lt;β&lt;\frac{3π}{2},$$ find</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -891,7 +891,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>$sin(α+β)sin(α+β)$</t>
+          <t>$$sin(α+β)$$</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -921,7 +921,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>$cos(α+β)cos(α+β)$</t>
+          <t>$$cos(α+β)$$</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -951,7 +951,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>$tan(α+β)tan(α+β)$</t>
+          <t>$$tan(α+β)$$</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -981,7 +981,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>$tan(α-β)tan(α-β)$</t>
+          <t>$$tan(α−β)$$</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Write $tan\frac{\pi }{9}tan\frac{\pi }{9}$ in terms of its cofunction.</t>
+          <t>Write $$tan\frac{π}{9}$$ in terms of its cofunction.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Verify the identity $sin(α+β)+sin(α-β)=2sinαcosβ.sin(α+β)+sin(α-β)=2sinαcosβ.$</t>
+          <t>Verify the identity $$sin(α+β)+sin(α−β)=2sinαcosβ.$$</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Verify the following identity. $\frac{sin(α-β)}{cosαcosβ}=tanα-tanβ\frac{sin(α-β)}{cosαcosβ}=tanα-tanβ$</t>
+          <t>Verify the following identity. $$\frac{sin(α−β)}{cosαcosβ}=tanα−tanβ$$</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Let $L_{1}L_{1}$ and $L_{2}L_{2}$ denote two non-vertical intersecting lines, and let $\theta \theta $ denote the acute angle between $L_{1}L_{1}$ and $L_{2}.L_{2}.$ See Figure 7 . Show that $tan\theta =\frac{m_{2}-m_{1}}{1+m_{1}m_{2}}tan\theta =\frac{m_{2}-m_{1}}{1+m_{1}m_{2}}$ where $m_{1}m_{1}$ and $m_{2}m_{2}$ are the slopes of $L_{1}L_{1}$ and $L_{2}L_{2}$ respectively. ( Hint: Use the fact that $tan\theta _{1}=m_{1}tan\theta _{1}=m_{1}$ and $tan\theta _{2}=m_{2}.tan\theta _{2}=m_{2}.$ ) Figure 7</t>
+          <t>Let $$L_{1}$$ and $$L_{2}$$ denote two non-vertical intersecting lines, and let $$θ$$ denote the acute angle between $$L_{1}$$ and $$L_{2}.$$ See Figure 7 . Show that $$tanθ=\frac{m_{2}−m_{1}}{1+m_{1}m_{2}}$$ where $$m_{1}$$ and $$m_{2}$$ are the slopes of $$L_{1}$$ and $$L_{2}$$ respectively. ( Hint: Use the fact that $$tanθ_{1}=m_{1}$$ and $$tanθ_{2}=m_{2}.$$ ) Figure 7</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>For a climbing wall, a guy-wire $RR$ is attached 47 feet high on a vertical pole. Added support is provided by another guy-wire $SS$ attached 40 feet above ground on the same pole. If the wires are attached to the ground 50 feet from the pole, find the angle $αα$ between the wires. See Figure 8 . Figure 8</t>
+          <t>For a climbing wall, a guy-wire $$R$$ is attached 47 feet high on a vertical pole. Added support is provided by another guy-wire $$S$$ attached 40 feet above ground on the same pole. If the wires are attached to the ground 50 feet from the pole, find the angle $$α$$ between the wires. See Figure 8 . Figure 8</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>

</xml_diff>

<commit_message>
modified gemini prompt to make data population more precise
</commit_message>
<xml_diff>
--- a/trig_examples.xlsx
+++ b/trig_examples.xlsx
@@ -534,7 +534,11 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/precalculus-2e/pages/7-2-sum-and-difference-identities</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
@@ -594,7 +598,11 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/precalculus-2e/pages/7-2-sum-and-difference-identities</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
@@ -658,7 +666,11 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/precalculus-2e/pages/7-2-sum-and-difference-identities</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
@@ -748,7 +760,11 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/precalculus-2e/pages/7-2-sum-and-difference-identities</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
@@ -808,7 +824,11 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/precalculus-2e/pages/7-2-sum-and-difference-identities</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
@@ -872,7 +892,11 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/precalculus-2e/pages/7-2-sum-and-difference-identities</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
@@ -1022,7 +1046,11 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/precalculus-2e/pages/7-2-sum-and-difference-identities</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
@@ -1082,7 +1110,11 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/precalculus-2e/pages/7-2-sum-and-difference-identities</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
@@ -1142,7 +1174,11 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/precalculus-2e/pages/7-2-sum-and-difference-identities</t>
+        </is>
+      </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
@@ -1202,7 +1238,11 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/precalculus-2e/pages/7-2-sum-and-difference-identities</t>
+        </is>
+      </c>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
@@ -1262,7 +1302,11 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/precalculus-2e/pages/7-2-sum-and-difference-identities</t>
+        </is>
+      </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>

</xml_diff>